<commit_message>
fix: validate legacy office rendering models
</commit_message>
<xml_diff>
--- a/public/fixtures/regressions/office-preview-showcase.xlsx
+++ b/public/fixtures/regressions/office-preview-showcase.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xy/Documents/Nexolyra/demo-user-space/office/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC96AAE1-5552-6D41-A2A8-BAA28F08E35F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1AEF291-1EC5-074A-9937-43EBAC8352DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1040" yWindow="620" windowWidth="16080" windowHeight="13920" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4180" yWindow="22280" windowWidth="29400" windowHeight="18440" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="Sparklines" sheetId="5" r:id="rId5"/>
     <sheet name="RTL &amp; CJK" sheetId="6" r:id="rId6"/>
     <sheet name="Reference" sheetId="7" state="hidden" r:id="rId7"/>
-    <sheet name="Native Objects" sheetId="8" r:id="rId8"/>
+    <sheet name="Native PivotTable and Slicer" sheetId="10" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Overview!$B$26:$F$30</definedName>
@@ -37,16 +37,20 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'RTL &amp; CJK'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">Sparklines!$1:$2</definedName>
     <definedName name="RegionalTotals">Data!$D$2:$D$13</definedName>
+    <definedName name="切片器_Format">#N/A</definedName>
     <definedName name="切片器_Region">#N/A</definedName>
+    <definedName name="切片器_Status">#N/A</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="39" r:id="rId9"/>
+    <pivotCache cacheId="0" r:id="rId9"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
       <x14:slicerCaches>
         <x14:slicerCache r:id="rId10"/>
+        <x14:slicerCache r:id="rId11"/>
+        <x14:slicerCache r:id="rId12"/>
       </x14:slicerCaches>
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
@@ -91,10 +95,9 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="2">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
   <futureMetadata name="XLDAPR" count="1">
     <bk>
@@ -105,30 +108,16 @@
       </extLst>
     </bk>
   </futureMetadata>
-  <futureMetadata name="XLRICHVALUE" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
   <cellMetadata count="1">
     <bk>
       <rc t="1" v="0"/>
     </bk>
   </cellMetadata>
-  <valueMetadata count="1">
-    <bk>
-      <rc t="2" v="0"/>
-    </bk>
-  </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="115">
   <si>
     <t>Spreadsheet Preview Showcase</t>
   </si>
@@ -483,9 +472,6 @@
     <t>SLIDE</t>
   </si>
   <si>
-    <t>S21 · Native PivotTable and Slicer</t>
-  </si>
-  <si>
     <t>Category</t>
   </si>
   <si>
@@ -497,6 +483,27 @@
   <si>
     <t>Total</t>
     <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>行标签</t>
+  </si>
+  <si>
+    <t>总计</t>
+  </si>
+  <si>
+    <t>列标签</t>
+  </si>
+  <si>
+    <t>求和项:Opens汇总</t>
+  </si>
+  <si>
+    <t>求和项:Saves汇总</t>
+  </si>
+  <si>
+    <t>平均值项:Fidelity汇总</t>
+  </si>
+  <si>
+    <t>交互筛选面板</t>
   </si>
 </sst>
 </file>
@@ -619,7 +626,7 @@
     </font>
     <font>
       <b/>
-      <sz val="18"/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="宋体"/>
       <family val="2"/>
@@ -665,7 +672,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF17324D"/>
+        <fgColor rgb="FF1D2330"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -757,7 +764,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -786,6 +793,13 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="30"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -801,9 +815,6 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -2496,25 +2507,25 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>63500</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>165819</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>1117600</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1074470</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>67206</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
-            <xdr:cNvPr id="2" name="PreviewRegionSlicer">
+            <xdr:cNvPr id="2" name="区域筛选">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1FB31971-126E-2E98-6649-727E15BA704A}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A3F6583C-E8FC-9C2B-BD2C-56D7BBEE8BF5}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2526,12 +2537,12 @@
           </xdr:xfrm>
           <a:graphic>
             <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
-              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="PreviewRegionSlicer"/>
+              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="区域筛选"/>
             </a:graphicData>
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -2541,8 +2552,164 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6858000" y="1143000"/>
-              <a:ext cx="2286000" cy="2413000"/>
+              <a:off x="15265400" y="482600"/>
+              <a:ext cx="1841500" cy="1841500"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="zh-CN" altLang="en-US" sz="1100"/>
+                <a:t>此形状代表切片器。Excel 2010 或更高版本支持切片器。
+如果形状是在较早版本的 Excel 中修改，或者工作簿是在 Excel 2003 或更早版本中保存，则无法使用切片器。</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1226870</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>165819</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>639664</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>67206</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="3" name="格式筛选">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7578F7EA-71C9-D4AF-B7CC-79B9D25821CA}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="格式筛选"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback xmlns="">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="17741900" y="482600"/>
+              <a:ext cx="2095500" cy="1841500"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="zh-CN" altLang="en-US" sz="1100"/>
+                <a:t>此形状代表切片器。Excel 2010 或更高版本支持切片器。
+如果形状是在较早版本的 Excel 中修改，或者工作簿是在 Excel 2003 或更早版本中保存，则无法使用切片器。</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>792064</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>165819</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>894520</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>116246</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="4" name="状态筛选">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{41D7737A-2D09-0AE2-7E9C-DB8C5A7C8FB6}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="状态筛选"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback xmlns="">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="15265400" y="2260600"/>
+              <a:ext cx="1841500" cy="1714500"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -2576,7 +2743,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Y X" refreshedDate="46225.661386805557" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="12" xr:uid="{F4FE4A09-ABFF-EF4F-8B6D-B7258715498C}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Y X" refreshedDate="46225.738048495368" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="12" xr:uid="{264EC25B-A91A-C147-8CA8-863504F12102}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:G13" sheet="Data"/>
   </cacheSource>
@@ -2618,7 +2785,7 @@
   </cacheFields>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition pivotCacheId="1461061910"/>
+      <x14:pivotCacheDefinition pivotCacheId="383411283"/>
     </ext>
   </extLst>
 </pivotCacheDefinition>
@@ -2738,30 +2905,30 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7395E7CF-89DB-5A43-ABAD-EB3F84768F6D}" name="PreviewCapabilityPivot" cacheId="39" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A4" firstHeaderRow="0" firstDataRow="0" firstDataCol="0"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9698208B-7886-0D40-B080-E37FCE9F6678}" name="数据透视表汇总" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:D6" firstHeaderRow="1" firstDataRow="3" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="7">
     <pivotField numFmtId="177" showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
       <items count="5">
-        <item x="2"/>
+        <item h="1" x="2"/>
         <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
+        <item h="1" x="1"/>
+        <item h="1" x="3"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField axis="axisCol" showAll="0">
       <items count="4">
-        <item x="0"/>
-        <item x="2"/>
+        <item h="1" x="0"/>
+        <item h="1" x="2"/>
         <item x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField dataField="1" showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
-    <pivotField numFmtId="176" showAll="0"/>
+    <pivotField dataField="1" numFmtId="176" showAll="0"/>
     <pivotField axis="axisPage" showAll="0">
       <items count="4">
         <item x="0"/>
@@ -2774,19 +2941,7 @@
   <rowFields count="1">
     <field x="1"/>
   </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
+  <rowItems count="1">
     <i t="grand">
       <x/>
     </i>
@@ -2795,41 +2950,24 @@
     <field x="2"/>
     <field x="-2"/>
   </colFields>
-  <colItems count="8">
-    <i>
-      <x/>
-      <x/>
-    </i>
-    <i r="1" i="1">
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="1"/>
-      <x/>
-    </i>
-    <i r="1" i="1">
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-      <x/>
-    </i>
-    <i r="1" i="1">
-      <x v="1"/>
-    </i>
+  <colItems count="3">
     <i t="grand">
       <x/>
     </i>
     <i t="grand" i="1">
-      <x/>
+      <x v="1"/>
+    </i>
+    <i t="grand" i="2">
+      <x v="2"/>
     </i>
   </colItems>
   <pageFields count="1">
-    <pageField fld="6" hier="-1"/>
+    <pageField fld="6" item="1" hier="-1"/>
   </pageFields>
-  <dataFields count="2">
-    <dataField name="Total opens" fld="3" baseField="0" baseItem="0"/>
-    <dataField name="Total saves" fld="4" baseField="0" baseItem="0"/>
+  <dataFields count="3">
+    <dataField name="求和项:Opens" fld="3" baseField="0" baseItem="0" numFmtId="3"/>
+    <dataField name="求和项:Saves" fld="4" baseField="0" baseItem="0" numFmtId="3"/>
+    <dataField name="平均值项:Fidelity" fld="5" subtotal="average" baseField="0" baseItem="0" numFmtId="176"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -2843,80 +2981,52 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
-<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
-  <global>
-    <keyFlags>
-      <key name="_Self">
-        <flag name="ExcludeFromFile" value="1"/>
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_DisplayString">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Flags">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Format">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_SubLabel">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Attribution">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Icon">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Display">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_CanonicalPropertyNames">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_ClassificationId">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-    </keyFlags>
-  </global>
-</rvTypesInfo>
+<file path=xl/slicerCaches/slicerCache1.xml><?xml version="1.0" encoding="utf-8"?>
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="切片器_Region" xr10:uid="{72271525-8EC4-ED48-A921-8743DFC80431}" sourceName="Region">
+  <pivotTables>
+    <pivotTable tabId="10" name="数据透视表汇总"/>
+  </pivotTables>
+  <data>
+    <tabular pivotCacheId="383411283">
+      <items count="4">
+        <i x="2" nd="1"/>
+        <i x="0" s="1" nd="1"/>
+        <i x="1" nd="1"/>
+        <i x="3" nd="1"/>
+      </items>
+    </tabular>
+  </data>
+</slicerCacheDefinition>
 </file>
 
-<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <rv s="0">
-    <v>8</v>
-    <v>8</v>
-    <v>7</v>
-    <v>7</v>
-  </rv>
-</rvData>
+<file path=xl/slicerCaches/slicerCache2.xml><?xml version="1.0" encoding="utf-8"?>
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="切片器_Format" xr10:uid="{D778362B-D99A-2649-8CE0-4528BDB6E301}" sourceName="Format">
+  <pivotTables>
+    <pivotTable tabId="10" name="数据透视表汇总"/>
+  </pivotTables>
+  <data>
+    <tabular pivotCacheId="383411283">
+      <items count="3">
+        <i x="2"/>
+        <i x="0" nd="1"/>
+        <i x="1" s="1" nd="1"/>
+      </items>
+    </tabular>
+  </data>
+</slicerCacheDefinition>
 </file>
 
-<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <s t="_error">
-    <k n="colOffset" t="i"/>
-    <k n="errorType" t="i"/>
-    <k n="rwOffset" t="i"/>
-    <k n="subType" t="i"/>
-  </s>
-</rvStructures>
-</file>
-
-<file path=xl/slicerCaches/slicerCache1.xml><?xml version="1.0" encoding="utf-8"?>
-<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="切片器_Region" xr10:uid="{C71BF13C-AB55-8B4E-AD35-B2F5E21F6970}" sourceName="Region">
+<file path=xl/slicerCaches/slicerCache3.xml><?xml version="1.0" encoding="utf-8"?>
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="切片器_Status" xr10:uid="{C0DD3CE1-39E8-C14E-8090-B59F25AFA904}" sourceName="Status">
   <pivotTables>
-    <pivotTable tabId="8" name="PreviewCapabilityPivot"/>
+    <pivotTable tabId="10" name="数据透视表汇总"/>
   </pivotTables>
   <data>
-    <tabular pivotCacheId="1461061910">
-      <items count="4">
-        <i x="2" s="1"/>
-        <i x="0" s="1"/>
-        <i x="1" s="1"/>
-        <i x="3" s="1"/>
+    <tabular pivotCacheId="383411283">
+      <items count="3">
+        <i x="0"/>
+        <i x="2" s="1" nd="1"/>
+        <i x="1" nd="1"/>
       </items>
     </tabular>
   </data>
@@ -2925,7 +3035,9 @@
 
 <file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
 <slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
-  <slicer name="PreviewRegionSlicer" xr10:uid="{406C9885-34FC-D14B-950C-53F1129D577F}" cache="切片器_Region" caption="Region" rowHeight="209550"/>
+  <slicer name="区域筛选" xr10:uid="{EA2EC87B-727C-2948-B66D-91C9A4ACAC5E}" cache="切片器_Region" caption="区域 Region" rowHeight="209550"/>
+  <slicer name="格式筛选" xr10:uid="{E779C762-06FF-4A44-BADD-22A224FA3979}" cache="切片器_Format" caption="格式 Format" rowHeight="209550"/>
+  <slicer name="状态筛选" xr10:uid="{F3395CC8-C9D1-3141-B1E1-9F3CE9F079F3}" cache="切片器_Status" caption="状态 Status" rowHeight="209550"/>
 </slicers>
 </file>
 
@@ -3281,86 +3393,86 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:12" ht="34" customHeight="1">
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
     </row>
     <row r="3" spans="2:12" ht="15">
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
     </row>
     <row r="5" spans="2:12" ht="18">
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="16"/>
-      <c r="J5" s="16"/>
-      <c r="K5" s="16"/>
-      <c r="L5" s="16"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="21"/>
+      <c r="I5" s="21"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="21"/>
+      <c r="L5" s="21"/>
     </row>
     <row r="6" spans="2:12" ht="15">
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19" t="s">
+      <c r="C6" s="24"/>
+      <c r="D6" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19" t="s">
+      <c r="E6" s="24"/>
+      <c r="F6" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19" t="s">
+      <c r="G6" s="24"/>
+      <c r="H6" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="I6" s="19"/>
+      <c r="I6" s="24"/>
     </row>
     <row r="7" spans="2:12" ht="24">
-      <c r="B7" s="20">
+      <c r="B7" s="25">
         <f>SUM(DataTable[Opens])</f>
         <v>2071</v>
       </c>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20">
+      <c r="C7" s="25"/>
+      <c r="D7" s="25">
         <f>SUM(DataTable[Saves])</f>
         <v>1110</v>
       </c>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20">
+      <c r="E7" s="25"/>
+      <c r="F7" s="25">
         <f>AVERAGE(DataTable[Fidelity])</f>
         <v>0.91500000000000015</v>
       </c>
-      <c r="G7" s="20"/>
-      <c r="H7" s="20">
+      <c r="G7" s="25"/>
+      <c r="H7" s="25">
         <f>COUNTIF(DataTable[Status],"Healthy")</f>
         <v>8</v>
       </c>
-      <c r="I7" s="20"/>
+      <c r="I7" s="25"/>
     </row>
     <row r="10" spans="2:12" ht="18">
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
     </row>
     <row r="11" spans="2:12" ht="15">
       <c r="B11" s="1" t="s">
@@ -3387,13 +3499,13 @@
       </c>
     </row>
     <row r="15" spans="2:12" ht="18">
-      <c r="B15" s="16" t="s">
+      <c r="B15" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="21"/>
     </row>
     <row r="16" spans="2:12" ht="15">
       <c r="B16" s="1" t="s">
@@ -3988,17 +4100,17 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" ht="30">
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
       <c r="G2" t="s">
+        <v>104</v>
+      </c>
+      <c r="H2" t="s">
         <v>105</v>
-      </c>
-      <c r="H2" t="s">
-        <v>106</v>
       </c>
       <c r="I2" t="s">
         <v>49</v>
@@ -4075,7 +4187,7 @@
         <v>56</v>
       </c>
       <c r="G6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H6">
         <v>4</v>
@@ -4098,7 +4210,7 @@
         <v>59</v>
       </c>
       <c r="G7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H7">
         <f>SUBTOTAL(109,TotalsDemo[Units])</f>
@@ -4202,12 +4314,12 @@
       </c>
     </row>
     <row r="16" spans="2:9" ht="28" customHeight="1">
-      <c r="B16" s="16" t="s">
+      <c r="B16" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="21"/>
     </row>
     <row r="18" spans="2:4" ht="42" customHeight="1">
       <c r="B18" s="14" t="s">
@@ -4395,18 +4507,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="30">
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
     </row>
     <row r="4" spans="2:11">
       <c r="B4" s="7" t="s">
@@ -4523,7 +4635,103 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{05C60535-1F16-4fd2-B633-F4F36F0B64E0}">
       <x14:sparklineGroups xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-        <x14:sparklineGroup displayEmptyCellsAs="gap" markers="1" xr2:uid="{00000000-0003-0000-0400-000008000000}">
+        <x14:sparklineGroup manualMax="0" manualMin="0" type="stacked" displayEmptyCellsAs="gap" xr2:uid="{00000000-0003-0000-0400-000000000000}">
+          <x14:colorSeries theme="4" tint="-0.499984740745262"/>
+          <x14:colorNegative theme="5"/>
+          <x14:colorAxis rgb="FF000000"/>
+          <x14:colorMarkers theme="4" tint="-0.499984740745262"/>
+          <x14:colorFirst theme="4" tint="0.39997558519241921"/>
+          <x14:colorLast theme="4" tint="0.39997558519241921"/>
+          <x14:colorHigh theme="4"/>
+          <x14:colorLow theme="4"/>
+          <x14:sparklines>
+            <x14:sparkline>
+              <xm:f>Sparklines!C7:H7</xm:f>
+              <xm:sqref>K7</xm:sqref>
+            </x14:sparkline>
+          </x14:sparklines>
+        </x14:sparklineGroup>
+        <x14:sparklineGroup manualMax="0" manualMin="0" type="column" displayEmptyCellsAs="gap" xr2:uid="{00000000-0003-0000-0400-000001000000}">
+          <x14:colorSeries theme="4" tint="-0.499984740745262"/>
+          <x14:colorNegative theme="5"/>
+          <x14:colorAxis rgb="FF000000"/>
+          <x14:colorMarkers theme="4" tint="-0.499984740745262"/>
+          <x14:colorFirst theme="4" tint="0.39997558519241921"/>
+          <x14:colorLast theme="4" tint="0.39997558519241921"/>
+          <x14:colorHigh theme="4"/>
+          <x14:colorLow theme="4"/>
+          <x14:sparklines>
+            <x14:sparkline>
+              <xm:f>Sparklines!C7:H7</xm:f>
+              <xm:sqref>J7</xm:sqref>
+            </x14:sparkline>
+          </x14:sparklines>
+        </x14:sparklineGroup>
+        <x14:sparklineGroup manualMax="0" manualMin="0" displayEmptyCellsAs="gap" markers="1" xr2:uid="{00000000-0003-0000-0400-000002000000}">
+          <x14:colorSeries theme="4" tint="-0.499984740745262"/>
+          <x14:colorNegative theme="5"/>
+          <x14:colorAxis rgb="FF000000"/>
+          <x14:colorMarkers theme="4" tint="-0.499984740745262"/>
+          <x14:colorFirst theme="4" tint="0.39997558519241921"/>
+          <x14:colorLast theme="4" tint="0.39997558519241921"/>
+          <x14:colorHigh theme="4"/>
+          <x14:colorLow theme="4"/>
+          <x14:sparklines>
+            <x14:sparkline>
+              <xm:f>Sparklines!C7:H7</xm:f>
+              <xm:sqref>I7</xm:sqref>
+            </x14:sparkline>
+          </x14:sparklines>
+        </x14:sparklineGroup>
+        <x14:sparklineGroup manualMax="0" manualMin="0" type="stacked" displayEmptyCellsAs="gap" xr2:uid="{00000000-0003-0000-0400-000003000000}">
+          <x14:colorSeries theme="4" tint="-0.499984740745262"/>
+          <x14:colorNegative theme="5"/>
+          <x14:colorAxis rgb="FF000000"/>
+          <x14:colorMarkers theme="4" tint="-0.499984740745262"/>
+          <x14:colorFirst theme="4" tint="0.39997558519241921"/>
+          <x14:colorLast theme="4" tint="0.39997558519241921"/>
+          <x14:colorHigh theme="4"/>
+          <x14:colorLow theme="4"/>
+          <x14:sparklines>
+            <x14:sparkline>
+              <xm:f>Sparklines!C6:H6</xm:f>
+              <xm:sqref>K6</xm:sqref>
+            </x14:sparkline>
+          </x14:sparklines>
+        </x14:sparklineGroup>
+        <x14:sparklineGroup manualMax="0" manualMin="0" type="column" displayEmptyCellsAs="gap" xr2:uid="{00000000-0003-0000-0400-000004000000}">
+          <x14:colorSeries theme="4" tint="-0.499984740745262"/>
+          <x14:colorNegative theme="5"/>
+          <x14:colorAxis rgb="FF000000"/>
+          <x14:colorMarkers theme="4" tint="-0.499984740745262"/>
+          <x14:colorFirst theme="4" tint="0.39997558519241921"/>
+          <x14:colorLast theme="4" tint="0.39997558519241921"/>
+          <x14:colorHigh theme="4"/>
+          <x14:colorLow theme="4"/>
+          <x14:sparklines>
+            <x14:sparkline>
+              <xm:f>Sparklines!C6:H6</xm:f>
+              <xm:sqref>J6</xm:sqref>
+            </x14:sparkline>
+          </x14:sparklines>
+        </x14:sparklineGroup>
+        <x14:sparklineGroup manualMax="0" manualMin="0" displayEmptyCellsAs="gap" markers="1" xr2:uid="{00000000-0003-0000-0400-000005000000}">
+          <x14:colorSeries theme="4" tint="-0.499984740745262"/>
+          <x14:colorNegative theme="5"/>
+          <x14:colorAxis rgb="FF000000"/>
+          <x14:colorMarkers theme="4" tint="-0.499984740745262"/>
+          <x14:colorFirst theme="4" tint="0.39997558519241921"/>
+          <x14:colorLast theme="4" tint="0.39997558519241921"/>
+          <x14:colorHigh theme="4"/>
+          <x14:colorLow theme="4"/>
+          <x14:sparklines>
+            <x14:sparkline>
+              <xm:f>Sparklines!C6:H6</xm:f>
+              <xm:sqref>I6</xm:sqref>
+            </x14:sparkline>
+          </x14:sparklines>
+        </x14:sparklineGroup>
+        <x14:sparklineGroup manualMax="0" manualMin="0" type="stacked" displayEmptyCellsAs="gap" xr2:uid="{00000000-0003-0000-0400-000006000000}">
           <x14:colorSeries theme="4" tint="-0.499984740745262"/>
           <x14:colorNegative theme="5"/>
           <x14:colorAxis rgb="FF000000"/>
@@ -4535,11 +4743,11 @@
           <x14:sparklines>
             <x14:sparkline>
               <xm:f>Sparklines!C5:H5</xm:f>
-              <xm:sqref>I5</xm:sqref>
+              <xm:sqref>K5</xm:sqref>
             </x14:sparkline>
           </x14:sparklines>
         </x14:sparklineGroup>
-        <x14:sparklineGroup type="column" displayEmptyCellsAs="gap" xr2:uid="{00000000-0003-0000-0400-000007000000}">
+        <x14:sparklineGroup manualMax="0" manualMin="0" type="column" displayEmptyCellsAs="gap" xr2:uid="{00000000-0003-0000-0400-000007000000}">
           <x14:colorSeries theme="4" tint="-0.499984740745262"/>
           <x14:colorNegative theme="5"/>
           <x14:colorAxis rgb="FF000000"/>
@@ -4555,7 +4763,7 @@
             </x14:sparkline>
           </x14:sparklines>
         </x14:sparklineGroup>
-        <x14:sparklineGroup type="stacked" displayEmptyCellsAs="gap" xr2:uid="{00000000-0003-0000-0400-000006000000}">
+        <x14:sparklineGroup manualMax="0" manualMin="0" displayEmptyCellsAs="gap" markers="1" xr2:uid="{00000000-0003-0000-0400-000008000000}">
           <x14:colorSeries theme="4" tint="-0.499984740745262"/>
           <x14:colorNegative theme="5"/>
           <x14:colorAxis rgb="FF000000"/>
@@ -4567,103 +4775,7 @@
           <x14:sparklines>
             <x14:sparkline>
               <xm:f>Sparklines!C5:H5</xm:f>
-              <xm:sqref>K5</xm:sqref>
-            </x14:sparkline>
-          </x14:sparklines>
-        </x14:sparklineGroup>
-        <x14:sparklineGroup displayEmptyCellsAs="gap" markers="1" xr2:uid="{00000000-0003-0000-0400-000005000000}">
-          <x14:colorSeries theme="4" tint="-0.499984740745262"/>
-          <x14:colorNegative theme="5"/>
-          <x14:colorAxis rgb="FF000000"/>
-          <x14:colorMarkers theme="4" tint="-0.499984740745262"/>
-          <x14:colorFirst theme="4" tint="0.39997558519241921"/>
-          <x14:colorLast theme="4" tint="0.39997558519241921"/>
-          <x14:colorHigh theme="4"/>
-          <x14:colorLow theme="4"/>
-          <x14:sparklines>
-            <x14:sparkline>
-              <xm:f>Sparklines!C6:H6</xm:f>
-              <xm:sqref>I6</xm:sqref>
-            </x14:sparkline>
-          </x14:sparklines>
-        </x14:sparklineGroup>
-        <x14:sparklineGroup type="column" displayEmptyCellsAs="gap" xr2:uid="{00000000-0003-0000-0400-000004000000}">
-          <x14:colorSeries theme="4" tint="-0.499984740745262"/>
-          <x14:colorNegative theme="5"/>
-          <x14:colorAxis rgb="FF000000"/>
-          <x14:colorMarkers theme="4" tint="-0.499984740745262"/>
-          <x14:colorFirst theme="4" tint="0.39997558519241921"/>
-          <x14:colorLast theme="4" tint="0.39997558519241921"/>
-          <x14:colorHigh theme="4"/>
-          <x14:colorLow theme="4"/>
-          <x14:sparklines>
-            <x14:sparkline>
-              <xm:f>Sparklines!C6:H6</xm:f>
-              <xm:sqref>J6</xm:sqref>
-            </x14:sparkline>
-          </x14:sparklines>
-        </x14:sparklineGroup>
-        <x14:sparklineGroup type="stacked" displayEmptyCellsAs="gap" xr2:uid="{00000000-0003-0000-0400-000003000000}">
-          <x14:colorSeries theme="4" tint="-0.499984740745262"/>
-          <x14:colorNegative theme="5"/>
-          <x14:colorAxis rgb="FF000000"/>
-          <x14:colorMarkers theme="4" tint="-0.499984740745262"/>
-          <x14:colorFirst theme="4" tint="0.39997558519241921"/>
-          <x14:colorLast theme="4" tint="0.39997558519241921"/>
-          <x14:colorHigh theme="4"/>
-          <x14:colorLow theme="4"/>
-          <x14:sparklines>
-            <x14:sparkline>
-              <xm:f>Sparklines!C6:H6</xm:f>
-              <xm:sqref>K6</xm:sqref>
-            </x14:sparkline>
-          </x14:sparklines>
-        </x14:sparklineGroup>
-        <x14:sparklineGroup displayEmptyCellsAs="gap" markers="1" xr2:uid="{00000000-0003-0000-0400-000002000000}">
-          <x14:colorSeries theme="4" tint="-0.499984740745262"/>
-          <x14:colorNegative theme="5"/>
-          <x14:colorAxis rgb="FF000000"/>
-          <x14:colorMarkers theme="4" tint="-0.499984740745262"/>
-          <x14:colorFirst theme="4" tint="0.39997558519241921"/>
-          <x14:colorLast theme="4" tint="0.39997558519241921"/>
-          <x14:colorHigh theme="4"/>
-          <x14:colorLow theme="4"/>
-          <x14:sparklines>
-            <x14:sparkline>
-              <xm:f>Sparklines!C7:H7</xm:f>
-              <xm:sqref>I7</xm:sqref>
-            </x14:sparkline>
-          </x14:sparklines>
-        </x14:sparklineGroup>
-        <x14:sparklineGroup type="column" displayEmptyCellsAs="gap" xr2:uid="{00000000-0003-0000-0400-000001000000}">
-          <x14:colorSeries theme="4" tint="-0.499984740745262"/>
-          <x14:colorNegative theme="5"/>
-          <x14:colorAxis rgb="FF000000"/>
-          <x14:colorMarkers theme="4" tint="-0.499984740745262"/>
-          <x14:colorFirst theme="4" tint="0.39997558519241921"/>
-          <x14:colorLast theme="4" tint="0.39997558519241921"/>
-          <x14:colorHigh theme="4"/>
-          <x14:colorLow theme="4"/>
-          <x14:sparklines>
-            <x14:sparkline>
-              <xm:f>Sparklines!C7:H7</xm:f>
-              <xm:sqref>J7</xm:sqref>
-            </x14:sparkline>
-          </x14:sparklines>
-        </x14:sparklineGroup>
-        <x14:sparklineGroup type="stacked" displayEmptyCellsAs="gap" xr2:uid="{00000000-0003-0000-0400-000000000000}">
-          <x14:colorSeries theme="4" tint="-0.499984740745262"/>
-          <x14:colorNegative theme="5"/>
-          <x14:colorAxis rgb="FF000000"/>
-          <x14:colorMarkers theme="4" tint="-0.499984740745262"/>
-          <x14:colorFirst theme="4" tint="0.39997558519241921"/>
-          <x14:colorLast theme="4" tint="0.39997558519241921"/>
-          <x14:colorHigh theme="4"/>
-          <x14:colorLow theme="4"/>
-          <x14:sparklines>
-            <x14:sparkline>
-              <xm:f>Sparklines!C7:H7</xm:f>
-              <xm:sqref>K7</xm:sqref>
+              <xm:sqref>I5</xm:sqref>
             </x14:sparkline>
           </x14:sparklines>
         </x14:sparklineGroup>
@@ -4687,49 +4799,49 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6" ht="20">
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="26" t="s">
         <v>94</v>
       </c>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
     </row>
     <row r="4" spans="2:6" ht="20">
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
     </row>
     <row r="6" spans="2:6" ht="17">
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
     </row>
     <row r="8" spans="2:6" ht="17">
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="C8" s="22"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="22"/>
-      <c r="F8" s="22"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
     </row>
     <row r="10" spans="2:6" ht="20">
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -4793,51 +4905,76 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25E14E3B-5071-8448-B833-957E0A27410D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF2C6098-9C5F-114A-89CE-188C39A43237}">
   <sheetPr>
-    <tabColor rgb="FF7B61FF"/>
+    <tabColor rgb="FF4472C4"/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:S11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="13" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="13" bestFit="1" customWidth="1"/>
-    <col min="8" max="11" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="22.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
-      <c r="A1" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" s="24"/>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="25" t="e" vm="1">
-        <v>#VALUE!</v>
+    <row r="1" spans="1:19" ht="24" customHeight="1">
+      <c r="A1" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" t="s">
+        <v>41</v>
+      </c>
+      <c r="N1" s="20"/>
+      <c r="O1" s="20"/>
+      <c r="P1" s="20"/>
+      <c r="Q1" s="20"/>
+      <c r="R1" s="20"/>
+      <c r="S1" s="20"/>
+    </row>
+    <row r="3" spans="1:19">
+      <c r="B3" s="16" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19">
+      <c r="B4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C4" t="s">
+        <v>112</v>
+      </c>
+      <c r="D4" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19">
+      <c r="A5" s="16" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19">
+      <c r="A6" s="17" t="s">
+        <v>109</v>
+      </c>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="19"/>
+    </row>
+    <row r="9" spans="1:19">
+      <c r="A9" s="20"/>
+    </row>
+    <row r="11" spans="1:19">
+      <c r="A11" s="20" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:H2"/>
-  </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId2"/>

</xml_diff>